<commit_message>
Check invoices and payments against more contract terms
Add contracts.py with code-decided checks of each vendor contract: unit price
vs the contract price list, invoice date vs contract period, payment date vs
credit term, cumulative invoiced amount vs contract ceiling, and contract
counterparty name vs the vendor master. Extend the TG Company samples with a
Bangkok Steel contract and two new TG transactions that plant one case of
each, update expected.json and regenerate the demo data.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RjVtj8pfYcMctujumP2iLZ
</commit_message>
<xml_diff>
--- a/pipeline/samples/tg_company/goods_receipts.xlsx
+++ b/pipeline/samples/tg_company/goods_receipts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -618,6 +618,46 @@
         <v>25000</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GR-2026-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PO-2026-010</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GR-2026-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PO-2026-011</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>32000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>